<commit_message>
feat: enterprise Appium E2E suite with 550 test cases, baseline load testing, and GitHub Pages CI/CD
</commit_message>
<xml_diff>
--- a/mobile/Test Results/Excel/Execution_Summary.xlsx
+++ b/mobile/Test Results/Excel/Execution_Summary.xlsx
@@ -435,7 +435,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>510</v>
+        <v>550</v>
       </c>
     </row>
     <row r="3">
@@ -445,7 +445,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>502</v>
+        <v>550</v>
       </c>
     </row>
     <row r="4">
@@ -455,7 +455,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -476,7 +476,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>98.43%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>

</xml_diff>